<commit_message>
add httpS to cannonical 93760300d6c48a88c3cdce72e4106e24efa84080
</commit_message>
<xml_diff>
--- a/ig/main/CodeSystem-competence-code-system.xlsx
+++ b/ig/main/CodeSystem-competence-code-system.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://interop.esante.gouv.fr/ig/documentation/CodeSystem/competence-code-system</t>
+    <t>https://interop.esante.gouv.fr/ig/documentation/CodeSystem/competence-code-system</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-05T12:31:03+00:00</t>
+    <t>2023-05-05T12:37:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>